<commit_message>
Update: Web interaktif 3 model soal + landing page harga Rp69.999 + Paket 1-5 PDF baru
</commit_message>
<xml_diff>
--- a/Quiz_Web_Bahasa_Indonesia_Paket_2.xlsx
+++ b/Quiz_Web_Bahasa_Indonesia_Paket_2.xlsx
@@ -436,19 +436,6 @@
   </sheetPr>
   <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -700,7 +687,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -724,8 +711,10 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="3" t="n">
-        <v>1</v>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>1, 3</t>
+        </is>
       </c>
       <c r="I6" s="3" t="n">
         <v>60</v>
@@ -801,27 +790,25 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Tegang dan penuh kekhawatiran warga kampung</t>
+          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Riuh, bangga, dan penuh decak kagum warga atas keberhasilan Rian</t>
+          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Sunyi senyap karena hujan badai yang sangat lebat</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Kecewa karena perahu robot tersangkut ranting pohon</t>
-        </is>
-      </c>
+          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="3" t="n">
-        <v>2</v>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="I8" s="3" t="n">
         <v>60</v>
@@ -1026,7 +1013,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1050,8 +1037,10 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="3" t="n">
-        <v>2</v>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>1, 3</t>
+        </is>
       </c>
       <c r="I13" s="3" t="n">
         <v>60</v>
@@ -1178,27 +1167,25 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Makanan pokok dan sayur-mayur</t>
+          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Lauk-pauk dan buah-buahan</t>
+          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Makanan pokok dan lauk-pauk</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Sayur-mayur dan buah-buahan</t>
-        </is>
-      </c>
+          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="3" t="n">
-        <v>1</v>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="I16" s="3" t="n">
         <v>60</v>
@@ -1312,7 +1299,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Checkbox</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1336,8 +1323,10 @@
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="3" t="n">
-        <v>1</v>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>1, 3</t>
+        </is>
       </c>
       <c r="I19" s="3" t="n">
         <v>60</v>
@@ -1409,27 +1398,25 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Rombongan wisatawan itu berlayar menyeberangi Selat Bali pada hari Minggu.</t>
+          <t>Pernyataan pertama berkaitan dengan konsep dasar materi ini.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Danau toba merupakan Danau vulkanik terbesar di Asia Tenggara.</t>
+          <t>Hasil perhitungan akhir bernilai lebih dari 50.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Ibu membeli buah Pisang ambon di pasar Tradisional.</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Setiap hari selasa, siswa kelas Enam memakai seragam pramuka.</t>
-        </is>
-      </c>
+          <t>Pernyataan ketiga bernilai salah berdasarkan analisis rumus.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="3" t="n">
-        <v>1</v>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="I21" s="3" t="n">
         <v>60</v>

</xml_diff>

<commit_message>
Add Paket 6-10 Worksheets: 10 new Matematika & Bahasa Indonesia .docx + .pdf files with 3 question variations
</commit_message>
<xml_diff>
--- a/Quiz_Web_Bahasa_Indonesia_Paket_2.xlsx
+++ b/Quiz_Web_Bahasa_Indonesia_Paket_2.xlsx
@@ -436,6 +436,19 @@
   </sheetPr>
   <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -682,39 +695,37 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Berdasarkan teks 'PLTS Terapung Cirata', manakah pernyataan yang merupakan FAKTA? (Pilih lebih dari satu)</t>
+          <t>Pernyataan berikut yang merupakan FAKTA yang dapat diverifikasi dari teks 'PLTS Terapung Cirata' adalah....</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PLTS Terapung Cirata dibangun di atas Waduk Cirata dengan kapasitas 192 MWp.</t>
+          <t>PLTS Terapung Cirata dibangun di atas permukaan waduk dengan kapasitas daya mencapai 192 MWp.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Semua PLTU batu bara di Indonesia harus ditutup segera.</t>
+          <t>Semua pembangkit listrik tenaga batu bara di Indonesia sebaiknya ditutup tahun depan.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Energi surya adalah energi terbarukan yang ramah lingkungan.</t>
+          <t>Energi matahari adalah satu-satunya sumber energi yang disukai masyarakat Jawa Barat.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>PLTS Cirata adalah yang paling indah di dunia.</t>
+          <t>Pemandangan panel surya di Waduk Cirata terlihat paling indah di seluruh dunia.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>1, 3</t>
-        </is>
+      <c r="H6" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>60</v>
@@ -722,7 +733,7 @@
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>A: Fakta (angka terukur 192 MWp, lokasi Waduk Cirata). B: Opini (harus ditutup = pendapat). C: Fakta (energi surya terbarukan &amp; ramah lingkungan). D: Opini (paling indah = subjektif). Jawaban benar: A, C.</t>
+          <t>Pilihan A menyajikan data faktual angka terukur: berkapasitas 192 MWp di Waduk Cirata. Pilihan B, C, dan D merupakan opini, saran subjektif, atau klaim berlebihan. Jawaban yang tepat adalah A.</t>
         </is>
       </c>
     </row>
@@ -780,7 +791,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Berdasarkan cerita robot Rian, tentukan kebenaran pernyataan berikut!</t>
+          <t>Suasana yang tercipta pada bagian akhir cerita saat robot buatan Rian berhasil bekerja adalah....</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -790,25 +801,27 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Suasana awal cerita cemas karena hujan badai.</t>
+          <t>Tegang dan penuh kekhawatiran warga kampung</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Suasana akhir cerita riah, bangga, dan penuh decak kagum warga.</t>
+          <t>Riuh, bangga, dan penuh decak kagum warga atas keberhasilan Rian</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Robot Rian gagal berfungsi dan membuat warga kecewa.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
+          <t>Sunyi senyap karena hujan badai yang sangat lebat</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Kecewa karena perahu robot tersangkut ranting pohon</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="H8" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>60</v>
@@ -816,7 +829,7 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>A: SALAH (awal cerita Rian membuat robot, bukan hujan badai). B: BENAR (teks: 'warga bertepuk tangan riuh, bangga, decak kagum'). C: SALAH (robot BERHASIL bekerja).</t>
+          <t>Di akhir cerita digambarkan: 'Warga kampung yang berkumpul di pinggir jalan bertepuk tangan riuh, kagum atas keuletan dan kecerdasan anak muda yang peduli pada lingkungannya tersebut.' Suasana yang tercipta adalah bangga dan kagum (Pilihan B).</t>
         </is>
       </c>
     </row>
@@ -1008,39 +1021,37 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Berdasarkan teks tradisi Marosok, tujuan penggunaan kain penutup saat tawar-menawar adalah.... (Pilih lebih dari satu)</t>
+          <t>Berdasarkan teks di atas, salah satu tujuan mulia dari penggunaan kain penutup saat tawar-menawar Marosok adalah....</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Menjaga kerahasiaan harga agar tidak memicu persaingan tidak sehat.</t>
+          <t>Menghangatkan tangan pembeli dan penjual dari cuaca dingin pegunungan</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Menghindarkan rasa malu pembeli jika harganya tidak terjangkau.</t>
+          <t>Menjaga kerahasiaan harga agar tidak memicu persaingan tidak sehat dan menghindarkan rasa malu pembeli</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Menghangatkan tangan saat berunding di cuaca dingin.</t>
+          <t>Menunjukkan status sosial dan kekayaan keluarga pembeli ternak</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Menunjukkan kekayaan pembeli melalui kain yang dipakai.</t>
+          <t>Menghitung jumlah uang kertas yang dibawa oleh calon pembeli</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
+      <c r="H13" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>60</v>
@@ -1048,7 +1059,7 @@
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>A &amp; B: Benar (teks: 'menjaga kerahasiaan harga agar tidak memicu persaingan tidak sehat dan menghindarkan rasa malu pembeli'). C: SALAH (bukan tujuan utama). D: SALAH (bukan untuk menunjukkan kekayaan). Jawaban benar: A, B.</t>
+          <t>Paragraf ketiga memaparkan filosofinya: menjaga privasi harga agar pembeli lain tidak tahu sehingga persaingan tidak sehat dapat dicegah, serta menjaga martabat/menghindarkan rasa malu pembeli jika tawarannya belum cocok (Pilihan B).</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1156,19 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Berdasarkan poster 'Gizi Seimbang Generasi Hebat', tentukan kebenaran!</t>
+          <t>Bacalah poster edukasi kesehatan berikut untuk menjawab soal nomor 15 dan 16!
+Panduan Gizi Seimbang Generasi Hebat: Gerakan 'Isi Piringku'
+Kementerian Kesehatan RI mengajak keluarga Indonesia menerapkan pedoman gizi seimbang sekali makan:
+- 2/3 dari setengah piring diisi MAKANAN POKOK (nasi, jagung, singkong, ubi) sebagai sumber energi utama.
+- 1/3 dari setengah piring diisi LAUK-PAUK (ikan, ayam, telur, tempe, tahu) kaya protein dan mineral.
+- 2/3 dari setengah piring lainnya diisi SAYUR-MAYUR segar aneka warna sumber serat dan vitamin.
+- 1/3 dari setengah piring lainnya diisi BUAH-BUAHAN lokal manis kaya antioksidan.
+Lengkapi piring sehatmu dengan 4 Pilar Gaya Hidup Sehat:
+(1) Cuci tangan pakai sabun dengan air mengalir sebelum dan sesudah makan.
+(2) Minum air putih minimal 8 gelas per hari untuk menjaga hidrasi tubuh.
+(3) Lakukan aktivitas fisik atau olahraga ringan minimal 30 menit setiap hari.
+(4) Pantau berat badan secara rutin setiap bulan.
+Berdasarkan panduan 'Isi Piringku' dalam poster edukasi di atas, kelompok makanan yang memiliki porsi seimbang sebesar 2/3 dari setengah piring adalah....</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1155,25 +1178,27 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Makanan pokok mengisi 2/3 dari setengah piring.</t>
+          <t>Makanan pokok dan sayur-mayur</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Sayur-mayur mengisi 1/3 dari setengah piring.</t>
+          <t>Lauk-pauk dan buah-buahan</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Lauk-pauk dan buah-buahan masing-masing mengisi 1/4 piring penuh.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr"/>
+          <t>Makanan pokok dan lauk-pauk</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Sayur-mayur dan buah-buahan</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="H16" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>60</v>
@@ -1181,7 +1206,7 @@
       <c r="J16" s="3" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>A: BENAR (poster: nasi 2/3 dari ½ piring). B: BENAR (sayur 1/3 dari ½ piring). C: SALAH (lauk 1/3 dari ½ piring, buah 1/3 dari ½ piring, BUKAN 1/4 piring penuh).</t>
+          <t>Dalam poster tertulis: Makanan pokok mengambil 2/3 dari setengah piring, dan sayur-mayur juga mengambil 2/3 dari setengah piring lainnya. Keduanya berimbang besar (Pilihan A).</t>
         </is>
       </c>
     </row>
@@ -1280,39 +1305,39 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Perhatikan pasangan kata berikut! (1) luas → memperluas, (2) panjang → memanjangkan, (3) dalam → memperdalam, (4) tinggi → memertinggikan. Manakah pasangan yang TEPAT? (Pilih lebih dari satu)</t>
+          <t>Perhatikan kalimat berikut!
+Pemerintah kota terus berupaya (luas) jalur hijau di sepanjang trotoar demi menyerap emisi kendaraan bermotor.
+Bentuk kata berimbuhan yang tepat untuk kata dalam tanda kurung agar membentuk kalimat yang efektif adalah....</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>luas → memperluas (tepat).</t>
+          <t>memperluas</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>panjang → memanjangkan (tepat).</t>
+          <t>meluaskan</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>dalam → memperdalam (tepat).</t>
+          <t>diperluas</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>tinggi → memertinggikan (tepat).</t>
+          <t>memperluaskan</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
+      <c r="H19" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>60</v>
@@ -1320,7 +1345,7 @@
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Semua pasangan tepat: luas-memperluas, panjang-memanjangkan, dalam-memperdalam, tinggi-memertinggikan (imbuhan memper- + kan pada kata sifat). Jawaban benar: A, B, C, D.</t>
+          <t>Kata dasar 'luas' merupakan kata sifat. Imbuhan pembentuk kata kerja yang menyatakan 'menjadikan lebih luas' adalah 'memper-' (memperluas). Bentuk 'memperluaskan' salah karena pleonasme (tumpang tindih afiks memper-...-kan pada kata sifat). Jadi kata yang baku dan tepat adalah 'memperluas' (Pilihan A).</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1399,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Tentukan kebenaran penulisan huruf kapital berikut!</t>
+          <t>Penulisan huruf kapital berikut yang tepat dan sesuai dengan kaidah EYD adalah....</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1384,25 +1409,27 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Selat Bali, hari Minggu → Penulisan BENAR.</t>
+          <t>Rombongan wisatawan itu berlayar menyeberangi Selat Bali pada hari Minggu.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Danau Toba, Gunung Merapi → Penulisan BENAR.</t>
+          <t>Danau toba merupakan Danau vulkanik terbesar di Asia Tenggara.</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Pisang Ambon, Pasar Tradisional → Penulisan BENAR.</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
+          <t>Ibu membeli buah Pisang ambon di pasar Tradisional.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Setiap hari selasa, siswa kelas Enam memakai seragam pramuka.</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="H21" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>60</v>
@@ -1410,7 +1437,12 @@
       <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>A: BENAR (Selat Bali = nama geografi, Minggu = hari). B: BENAR (Danau Toba, Gunung Merapi = nama geografi). C: SALAH (pisang ambon = jenis buah, bukan nama diri → huruf kecil; pasar tradisional = umum, bukan nama diri).</t>
+          <t>Analisis ejaan:
+- Pilihan A: BENAR. Nama diri geografi (Selat Bali) huruf kapital, nama hari (Minggu) huruf kapital.
+- Pilihan B: salah, harusnya Danau Toba (T kapital), 'danau' pada danau vulkanik huruf kecil.
+- Pilihan C: salah, pisang ambon adalah nama jenis (bukan nama diri), jadi p dan a huruf kecil.
+- Pilihan D: salah, selasa harus kapital (Selasa), enam huruf kecil.
+Jadi kalimat yang benar adalah A.</t>
         </is>
       </c>
     </row>

</xml_diff>